<commit_message>
Semana 4: firmware de pruebas IMU/homing, evidencias de banco y ANSYS, avance de arquitectura de referencia absoluta
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estado-del-arte/SIMULADOR DE MARCHA/LIBRA_Config_Impresion_y_Calculo_Material.xlsx
+++ b/Estado-del-arte/SIMULADOR DE MARCHA/LIBRA_Config_Impresion_y_Calculo_Material.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aLESS\Documents\LIBRA\Estado-del-arte\SIMULADOR DE MARCHA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440A9D3E-D0E2-4CAB-B388-C7A798C8364F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79A9748-E241-441B-9274-4DB3D9278856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="107">
   <si>
     <t>LIBRA — Configuración de impresión recomendada (bracket pylon)</t>
   </si>
@@ -497,16 +497,6 @@
   </cellStyleXfs>
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -531,7 +521,17 @@
     <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,169 +806,169 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -993,151 +993,151 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
     </row>
     <row r="5" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="8">
         <v>1.24</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="8">
         <v>2.2999999999999998</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="8">
         <v>0.36</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="8">
         <v>20</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="8">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="8">
         <v>1.27</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="8">
         <v>1.8</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="8">
         <v>0.38</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="8">
         <v>22</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="8">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="8">
         <v>1.04</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="8">
         <v>2</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="8">
         <v>0.35</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="8">
         <v>16</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="8">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="8">
         <v>1.02</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="8">
         <v>1.5</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="8">
         <v>0.39</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="8">
         <v>30</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="8">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="8">
         <v>1.2</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="8">
         <v>3</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="8">
         <v>0.35</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="8">
         <v>28</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="8">
         <v>38</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1162,85 +1162,85 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
     </row>
     <row r="5" spans="2:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="8">
         <v>2</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="8">
         <v>1.5</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="9" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="8">
         <v>1.8</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="8">
         <v>1.4</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="9" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="8">
         <v>1.6</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="8">
         <v>1.3</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="8">
         <v>1.5</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="8">
         <v>1.3</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1280,950 +1280,960 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1" t="s">
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1" t="s">
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1" t="s">
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
     </row>
     <row r="6" spans="2:21" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="L6" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="M6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="N6" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q6" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="R6" s="7" t="s">
+      <c r="R6" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="S6" s="7" t="s">
+      <c r="S6" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="T6" s="7" t="s">
+      <c r="T6" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="U6" s="7" t="s">
+      <c r="U6" s="3" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="11">
         <v>60</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="10">
         <v>179.91</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="16">
         <v>223.8</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="12">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C7,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v>1.27</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="12">
         <f t="shared" ref="I7:I18" si="0">IFERROR(IF(AND(F7&lt;&gt;"",G7&lt;&gt;"",G7&lt;&gt;0),F7/G7,IF(E7&lt;&gt;"",(E7/100)*H7,"")),"")</f>
         <v>0.80388739946380694</v>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="12">
         <f t="shared" ref="J7:J18" si="1">IFERROR(I7/H7,"")</f>
         <v>0.63298220430221019</v>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="12">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D7,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v>2</v>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="12">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D7,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v>1.5</v>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="12">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C7,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v>0.38</v>
       </c>
-      <c r="N7" s="16">
+      <c r="N7" s="12">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C7,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J7,K7),"")</f>
         <v>0.72119964773391287</v>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="13">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C7,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J7,L7),"")</f>
         <v>11.079239010621558</v>
       </c>
-      <c r="P7" s="17">
+      <c r="P7" s="13">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C7,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J7,L7),"")</f>
         <v>15.108053196302125</v>
       </c>
-      <c r="Q7" s="18">
+      <c r="Q7" s="14">
         <f t="shared" ref="Q7:Q18" si="2">IFERROR(I7*1000,"")</f>
         <v>803.8873994638069</v>
       </c>
-      <c r="R7" s="21">
+      <c r="R7" s="17">
         <f t="shared" ref="R7:R18" si="3">IFERROR(N7*1000000000,"")</f>
         <v>721199647.73391283</v>
       </c>
-      <c r="S7" s="16">
+      <c r="S7" s="12">
         <f t="shared" ref="S7:S18" si="4">IFERROR(M7,"")</f>
         <v>0.38</v>
       </c>
-      <c r="T7" s="21">
+      <c r="T7" s="17">
         <f t="shared" ref="T7:T18" si="5">IFERROR(O7*1000000,"")</f>
         <v>11079239.010621559</v>
       </c>
-      <c r="U7" s="21">
+      <c r="U7" s="17">
         <f t="shared" ref="U7:U18" si="6">IFERROR(P7*1000000,"")</f>
         <v>15108053.196302125</v>
       </c>
     </row>
     <row r="8" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="16" t="str">
+      <c r="C8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="11">
+        <v>60</v>
+      </c>
+      <c r="F8" s="10">
+        <v>164.88</v>
+      </c>
+      <c r="G8" s="16">
+        <v>223.8</v>
+      </c>
+      <c r="H8" s="12">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C8,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="16" t="str">
+        <v>1.2</v>
+      </c>
+      <c r="I8" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="16" t="str">
+        <v>0.7367292225201072</v>
+      </c>
+      <c r="J8" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16" t="str">
+        <v>0.613941018766756</v>
+      </c>
+      <c r="K8" s="12">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D8,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
-        <v/>
-      </c>
-      <c r="L8" s="16" t="str">
+        <v>2</v>
+      </c>
+      <c r="L8" s="12">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D8,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="16" t="str">
+        <v>1.5</v>
+      </c>
+      <c r="M8" s="12">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C8,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
-        <v/>
-      </c>
-      <c r="N8" s="16" t="str">
+        <v>0.35</v>
+      </c>
+      <c r="N8" s="12">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C8,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J8,K8),"")</f>
-        <v/>
-      </c>
-      <c r="O8" s="17" t="str">
+        <v>1.1307707235730868</v>
+      </c>
+      <c r="O8" s="13">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C8,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J8,L8),"")</f>
-        <v/>
-      </c>
-      <c r="P8" s="17" t="str">
+        <v>13.469392457683616</v>
+      </c>
+      <c r="P8" s="13">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C8,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J8,L8),"")</f>
-        <v/>
-      </c>
-      <c r="Q8" s="18" t="str">
+        <v>18.279889763999194</v>
+      </c>
+      <c r="Q8" s="14">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="R8" s="19" t="str">
+        <v>736.72922252010721</v>
+      </c>
+      <c r="R8" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="S8" s="16" t="str">
+        <v>1130770723.5730867</v>
+      </c>
+      <c r="S8" s="12">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="T8" s="19" t="str">
+        <v>0.35</v>
+      </c>
+      <c r="T8" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="U8" s="19" t="str">
+        <v>13469392.457683617</v>
+      </c>
+      <c r="U8" s="15">
         <f t="shared" si="6"/>
-        <v/>
+        <v>18279889.763999194</v>
       </c>
     </row>
     <row r="9" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="16" t="str">
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C9,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I9" s="16" t="str">
+      <c r="I9" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J9" s="16" t="str">
+      <c r="J9" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K9" s="16" t="str">
+      <c r="K9" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D9,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L9" s="16" t="str">
+      <c r="L9" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D9,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M9" s="16" t="str">
+      <c r="M9" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C9,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N9" s="16" t="str">
+      <c r="N9" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C9,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J9,K9),"")</f>
         <v/>
       </c>
-      <c r="O9" s="17" t="str">
+      <c r="O9" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C9,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J9,L9),"")</f>
         <v/>
       </c>
-      <c r="P9" s="17" t="str">
+      <c r="P9" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C9,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J9,L9),"")</f>
         <v/>
       </c>
-      <c r="Q9" s="18" t="str">
+      <c r="Q9" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R9" s="19" t="str">
+      <c r="R9" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S9" s="16" t="str">
+      <c r="S9" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T9" s="19" t="str">
+      <c r="T9" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U9" s="19" t="str">
+      <c r="U9" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="10" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="16" t="str">
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C10,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I10" s="16" t="str">
+      <c r="I10" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J10" s="16" t="str">
+      <c r="J10" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K10" s="16" t="str">
+      <c r="K10" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D10,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L10" s="16" t="str">
+      <c r="L10" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D10,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M10" s="16" t="str">
+      <c r="M10" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C10,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N10" s="16" t="str">
+      <c r="N10" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C10,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J10,K10),"")</f>
         <v/>
       </c>
-      <c r="O10" s="17" t="str">
+      <c r="O10" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C10,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J10,L10),"")</f>
         <v/>
       </c>
-      <c r="P10" s="17" t="str">
+      <c r="P10" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C10,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J10,L10),"")</f>
         <v/>
       </c>
-      <c r="Q10" s="18" t="str">
+      <c r="Q10" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R10" s="19" t="str">
+      <c r="R10" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S10" s="16" t="str">
+      <c r="S10" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T10" s="19" t="str">
+      <c r="T10" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U10" s="19" t="str">
+      <c r="U10" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="11" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="16" t="str">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C11,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I11" s="16" t="str">
+      <c r="I11" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J11" s="16" t="str">
+      <c r="J11" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K11" s="16" t="str">
+      <c r="K11" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D11,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L11" s="16" t="str">
+      <c r="L11" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D11,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M11" s="16" t="str">
+      <c r="M11" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C11,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N11" s="16" t="str">
+      <c r="N11" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C11,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J11,K11),"")</f>
         <v/>
       </c>
-      <c r="O11" s="17" t="str">
+      <c r="O11" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C11,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J11,L11),"")</f>
         <v/>
       </c>
-      <c r="P11" s="17" t="str">
+      <c r="P11" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C11,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J11,L11),"")</f>
         <v/>
       </c>
-      <c r="Q11" s="18" t="str">
+      <c r="Q11" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R11" s="19" t="str">
+      <c r="R11" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S11" s="16" t="str">
+      <c r="S11" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T11" s="19" t="str">
+      <c r="T11" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U11" s="19" t="str">
+      <c r="U11" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="12" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="16" t="str">
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C12,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I12" s="16" t="str">
+      <c r="I12" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J12" s="16" t="str">
+      <c r="J12" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K12" s="16" t="str">
+      <c r="K12" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D12,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L12" s="16" t="str">
+      <c r="L12" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D12,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M12" s="16" t="str">
+      <c r="M12" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C12,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N12" s="16" t="str">
+      <c r="N12" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C12,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J12,K12),"")</f>
         <v/>
       </c>
-      <c r="O12" s="17" t="str">
+      <c r="O12" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C12,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J12,L12),"")</f>
         <v/>
       </c>
-      <c r="P12" s="17" t="str">
+      <c r="P12" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C12,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J12,L12),"")</f>
         <v/>
       </c>
-      <c r="Q12" s="18" t="str">
+      <c r="Q12" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R12" s="19" t="str">
+      <c r="R12" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S12" s="16" t="str">
+      <c r="S12" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T12" s="19" t="str">
+      <c r="T12" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U12" s="19" t="str">
+      <c r="U12" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="13" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="16" t="str">
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C13,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I13" s="16" t="str">
+      <c r="I13" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J13" s="16" t="str">
+      <c r="J13" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K13" s="16" t="str">
+      <c r="K13" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D13,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L13" s="16" t="str">
+      <c r="L13" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D13,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M13" s="16" t="str">
+      <c r="M13" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C13,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N13" s="16" t="str">
+      <c r="N13" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C13,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J13,K13),"")</f>
         <v/>
       </c>
-      <c r="O13" s="17" t="str">
+      <c r="O13" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C13,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J13,L13),"")</f>
         <v/>
       </c>
-      <c r="P13" s="17" t="str">
+      <c r="P13" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C13,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J13,L13),"")</f>
         <v/>
       </c>
-      <c r="Q13" s="18" t="str">
+      <c r="Q13" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R13" s="19" t="str">
+      <c r="R13" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S13" s="16" t="str">
+      <c r="S13" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T13" s="19" t="str">
+      <c r="T13" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U13" s="19" t="str">
+      <c r="U13" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="14" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="16" t="str">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C14,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I14" s="16" t="str">
+      <c r="I14" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J14" s="16" t="str">
+      <c r="J14" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K14" s="16" t="str">
+      <c r="K14" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D14,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L14" s="16" t="str">
+      <c r="L14" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D14,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M14" s="16" t="str">
+      <c r="M14" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C14,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N14" s="16" t="str">
+      <c r="N14" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C14,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J14,K14),"")</f>
         <v/>
       </c>
-      <c r="O14" s="17" t="str">
+      <c r="O14" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C14,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J14,L14),"")</f>
         <v/>
       </c>
-      <c r="P14" s="17" t="str">
+      <c r="P14" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C14,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J14,L14),"")</f>
         <v/>
       </c>
-      <c r="Q14" s="18" t="str">
+      <c r="Q14" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R14" s="19" t="str">
+      <c r="R14" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S14" s="16" t="str">
+      <c r="S14" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T14" s="19" t="str">
+      <c r="T14" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U14" s="19" t="str">
+      <c r="U14" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="15" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="16" t="str">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C15,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I15" s="16" t="str">
+      <c r="I15" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J15" s="16" t="str">
+      <c r="J15" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K15" s="16" t="str">
+      <c r="K15" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D15,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L15" s="16" t="str">
+      <c r="L15" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D15,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M15" s="16" t="str">
+      <c r="M15" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C15,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N15" s="16" t="str">
+      <c r="N15" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C15,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J15,K15),"")</f>
         <v/>
       </c>
-      <c r="O15" s="17" t="str">
+      <c r="O15" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C15,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J15,L15),"")</f>
         <v/>
       </c>
-      <c r="P15" s="17" t="str">
+      <c r="P15" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C15,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J15,L15),"")</f>
         <v/>
       </c>
-      <c r="Q15" s="18" t="str">
+      <c r="Q15" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R15" s="19" t="str">
+      <c r="R15" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S15" s="16" t="str">
+      <c r="S15" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T15" s="19" t="str">
+      <c r="T15" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U15" s="19" t="str">
+      <c r="U15" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="16" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="16" t="str">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C16,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I16" s="16" t="str">
+      <c r="I16" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J16" s="16" t="str">
+      <c r="J16" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K16" s="16" t="str">
+      <c r="K16" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D16,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L16" s="16" t="str">
+      <c r="L16" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D16,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M16" s="16" t="str">
+      <c r="M16" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C16,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N16" s="16" t="str">
+      <c r="N16" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C16,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J16,K16),"")</f>
         <v/>
       </c>
-      <c r="O16" s="17" t="str">
+      <c r="O16" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C16,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J16,L16),"")</f>
         <v/>
       </c>
-      <c r="P16" s="17" t="str">
+      <c r="P16" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C16,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J16,L16),"")</f>
         <v/>
       </c>
-      <c r="Q16" s="18" t="str">
+      <c r="Q16" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R16" s="19" t="str">
+      <c r="R16" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S16" s="16" t="str">
+      <c r="S16" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T16" s="19" t="str">
+      <c r="T16" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U16" s="19" t="str">
+      <c r="U16" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="17" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="16" t="str">
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C17,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I17" s="16" t="str">
+      <c r="I17" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J17" s="16" t="str">
+      <c r="J17" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K17" s="16" t="str">
+      <c r="K17" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D17,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L17" s="16" t="str">
+      <c r="L17" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D17,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M17" s="16" t="str">
+      <c r="M17" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C17,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N17" s="16" t="str">
+      <c r="N17" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C17,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J17,K17),"")</f>
         <v/>
       </c>
-      <c r="O17" s="17" t="str">
+      <c r="O17" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C17,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J17,L17),"")</f>
         <v/>
       </c>
-      <c r="P17" s="17" t="str">
+      <c r="P17" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C17,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J17,L17),"")</f>
         <v/>
       </c>
-      <c r="Q17" s="18" t="str">
+      <c r="Q17" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R17" s="19" t="str">
+      <c r="R17" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S17" s="16" t="str">
+      <c r="S17" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T17" s="19" t="str">
+      <c r="T17" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U17" s="19" t="str">
+      <c r="U17" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="18" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="16" t="str">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C18,'Propiedades Base'!$B$6:$B$10,0),2),"")</f>
         <v/>
       </c>
-      <c r="I18" s="16" t="str">
+      <c r="I18" s="12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J18" s="16" t="str">
+      <c r="J18" s="12" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K18" s="16" t="str">
+      <c r="K18" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D18,'Patrones Infill'!$B$6:$B$9,0),2),"")</f>
         <v/>
       </c>
-      <c r="L18" s="16" t="str">
+      <c r="L18" s="12" t="str">
         <f>IFERROR(INDEX('Patrones Infill'!$B$6:$D$9,MATCH(D18,'Patrones Infill'!$B$6:$B$9,0),3),"")</f>
         <v/>
       </c>
-      <c r="M18" s="16" t="str">
+      <c r="M18" s="12" t="str">
         <f>IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C18,'Propiedades Base'!$B$6:$B$10,0),4),"")</f>
         <v/>
       </c>
-      <c r="N18" s="16" t="str">
+      <c r="N18" s="12" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C18,'Propiedades Base'!$B$6:$B$10,0),3),"")*POWER(J18,K18),"")</f>
         <v/>
       </c>
-      <c r="O18" s="17" t="str">
+      <c r="O18" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C18,'Propiedades Base'!$B$6:$B$10,0),5),"")*POWER(J18,L18),"")</f>
         <v/>
       </c>
-      <c r="P18" s="17" t="str">
+      <c r="P18" s="13" t="str">
         <f>IFERROR(IFERROR(INDEX('Propiedades Base'!$B$6:$G$10,MATCH(C18,'Propiedades Base'!$B$6:$B$10,0),6),"")*POWER(J18,L18),"")</f>
         <v/>
       </c>
-      <c r="Q18" s="18" t="str">
+      <c r="Q18" s="14" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="R18" s="19" t="str">
+      <c r="R18" s="15" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="S18" s="16" t="str">
+      <c r="S18" s="12" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="T18" s="19" t="str">
+      <c r="T18" s="15" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U18" s="19" t="str">
+      <c r="U18" s="15" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="21" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="6" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="22" spans="2:21" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="18"/>
+      <c r="M22" s="18"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2235,8 +2245,8 @@
     <mergeCell ref="Q5:U5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">

</xml_diff>